<commit_message>
feat: update data test
</commit_message>
<xml_diff>
--- a/data/data_test.xlsx
+++ b/data/data_test.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="25601"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Test\script-test\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{0875D6BE-8C85-4AD5-A229-C8F4C1CA2EA4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3D37CC93-7C75-42D6-AB59-45EA633E4A4A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20640" windowHeight="11160" xr2:uid="{8FAFAB84-7321-4A60-AD43-F6BDBFF31D96}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{8FAFAB84-7321-4A60-AD43-F6BDBFF31D96}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="95" uniqueCount="47">
   <si>
     <t>Test Case ID</t>
   </si>
@@ -42,9 +42,6 @@
     <t>Test Case Description</t>
   </si>
   <si>
-    <t>Input Data</t>
-  </si>
-  <si>
     <t>Result</t>
   </si>
   <si>
@@ -52,13 +49,139 @@
   </si>
   <si>
     <t>Actualy result</t>
+  </si>
+  <si>
+    <t>Test login with valid credentials</t>
+  </si>
+  <si>
+    <t>Test login with a non-existent email</t>
+  </si>
+  <si>
+    <t>Test login with an incorrect email</t>
+  </si>
+  <si>
+    <t>Test login with an incorrect password</t>
+  </si>
+  <si>
+    <t>Test login with a missing email</t>
+  </si>
+  <si>
+    <t>Test login with a missing password</t>
+  </si>
+  <si>
+    <t>Username</t>
+  </si>
+  <si>
+    <t>Password</t>
+  </si>
+  <si>
+    <t>Platform</t>
+  </si>
+  <si>
+    <t>APP</t>
+  </si>
+  <si>
+    <t>testuser@example.com</t>
+  </si>
+  <si>
+    <t>Password123</t>
+  </si>
+  <si>
+    <t>nonexistent@example.com</t>
+  </si>
+  <si>
+    <t>testuser1@example.com</t>
+  </si>
+  <si>
+    <t>WrongPassword</t>
+  </si>
+  <si>
+    <t>[Login-11]</t>
+  </si>
+  <si>
+    <t>[Login-12]</t>
+  </si>
+  <si>
+    <t>[Login-13]</t>
+  </si>
+  <si>
+    <t>[Login-14]</t>
+  </si>
+  <si>
+    <t>[Login-15]</t>
+  </si>
+  <si>
+    <t>[Login-16]</t>
+  </si>
+  <si>
+    <t>[Login-17]</t>
+  </si>
+  <si>
+    <t>[Login-18]</t>
+  </si>
+  <si>
+    <t>[Login-19]</t>
+  </si>
+  <si>
+    <t>Test login with an overly long email</t>
+  </si>
+  <si>
+    <t>Test login with an overly long password</t>
+  </si>
+  <si>
+    <t>Test login with both email and password missing</t>
+  </si>
+  <si>
+    <t>a_very_long_email_address_that_exceeds_the_limit_of_100_characters_to_test_the_boundary@example.com</t>
+  </si>
+  <si>
+    <t>Password12345678912345678912345678912345678901234567890123456789</t>
+  </si>
+  <si>
+    <t>WEB</t>
+  </si>
+  <si>
+    <t>[Login-21]</t>
+  </si>
+  <si>
+    <t>Test login with an incorrectly formatted email</t>
+  </si>
+  <si>
+    <t>testuserexample.com</t>
+  </si>
+  <si>
+    <t>[Login-22]</t>
+  </si>
+  <si>
+    <t>[Login-23]</t>
+  </si>
+  <si>
+    <t>[Login-24]</t>
+  </si>
+  <si>
+    <t>[Login-25]</t>
+  </si>
+  <si>
+    <t>[Login-26]</t>
+  </si>
+  <si>
+    <t>[Login-27]</t>
+  </si>
+  <si>
+    <t>[Login-28]</t>
+  </si>
+  <si>
+    <t>[Login-29]</t>
+  </si>
+  <si>
+    <t>[Login-30]</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -79,16 +202,48 @@
       <name val="Times New Roman"/>
       <family val="1"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Tahoma"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Tahoma"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -111,26 +266,121 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFCCCCCC"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -443,160 +693,427 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A869C040-2518-4127-9479-80AA9CA67B0C}">
-  <dimension ref="A1:F16"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:H20"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="11.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="20.140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="13.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="8.5703125" style="1" customWidth="1"/>
-    <col min="7" max="16384" width="9.140625" style="1"/>
+    <col min="1" max="1" width="11.5546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="28.88671875" style="1" customWidth="1"/>
+    <col min="3" max="3" width="35.5546875" style="1" customWidth="1"/>
+    <col min="4" max="4" width="25.6640625" style="1" customWidth="1"/>
+    <col min="5" max="5" width="23.88671875" style="1" customWidth="1"/>
+    <col min="6" max="6" width="18.33203125" style="1" customWidth="1"/>
+    <col min="7" max="16384" width="9.109375" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="28.5" x14ac:dyDescent="0.25">
-      <c r="A1" s="4" t="s">
+    <row r="1" spans="1:8" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="B1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="C1" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="H1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="E1" s="4" t="s">
+    </row>
+    <row r="2" spans="1:8" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="B2" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="F1" s="4" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2" s="3"/>
-      <c r="B2" s="3"/>
-      <c r="C2" s="3"/>
-      <c r="D2" s="3"/>
-      <c r="E2" s="3"/>
-      <c r="F2" s="3"/>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" s="3"/>
-      <c r="B3" s="3"/>
-      <c r="C3" s="3"/>
-      <c r="D3" s="3"/>
-      <c r="E3" s="3"/>
-      <c r="F3" s="3"/>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A4" s="3"/>
-      <c r="B4" s="3"/>
-      <c r="C4" s="3"/>
-      <c r="D4" s="3"/>
-      <c r="E4" s="3"/>
-      <c r="F4" s="3"/>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A5" s="3"/>
-      <c r="B5" s="3"/>
-      <c r="C5" s="3"/>
-      <c r="D5" s="3"/>
-      <c r="E5" s="3"/>
-      <c r="F5" s="3"/>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A6" s="3"/>
-      <c r="B6" s="3"/>
-      <c r="C6" s="3"/>
-      <c r="D6" s="3"/>
-      <c r="E6" s="3"/>
-      <c r="F6" s="3"/>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A7" s="3"/>
-      <c r="B7" s="3"/>
-      <c r="C7" s="3"/>
-      <c r="D7" s="3"/>
-      <c r="E7" s="3"/>
-      <c r="F7" s="3"/>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A8" s="3"/>
-      <c r="B8" s="3"/>
-      <c r="C8" s="3"/>
-      <c r="D8" s="3"/>
-      <c r="E8" s="3"/>
-      <c r="F8" s="3"/>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A9" s="3"/>
-      <c r="B9" s="3"/>
-      <c r="C9" s="3"/>
-      <c r="D9" s="3"/>
-      <c r="E9" s="3"/>
-      <c r="F9" s="3"/>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A10" s="3"/>
-      <c r="B10" s="3"/>
-      <c r="C10" s="3"/>
-      <c r="D10" s="3"/>
-      <c r="E10" s="3"/>
-      <c r="F10" s="3"/>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A11" s="3"/>
-      <c r="B11" s="3"/>
-      <c r="C11" s="3"/>
-      <c r="D11" s="3"/>
-      <c r="E11" s="3"/>
-      <c r="F11" s="3"/>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A12" s="3"/>
-      <c r="B12" s="3"/>
-      <c r="C12" s="3"/>
-      <c r="D12" s="3"/>
-      <c r="E12" s="3"/>
-      <c r="F12" s="3"/>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A13" s="3"/>
-      <c r="B13" s="3"/>
-      <c r="C13" s="3"/>
-      <c r="D13" s="3"/>
-      <c r="E13" s="3"/>
-      <c r="F13" s="3"/>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A14" s="3"/>
-      <c r="B14" s="3"/>
-      <c r="C14" s="3"/>
-      <c r="D14" s="3"/>
-      <c r="E14" s="3"/>
-      <c r="F14" s="3"/>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A15" s="2"/>
-      <c r="B15" s="2"/>
-      <c r="C15" s="2"/>
-      <c r="D15" s="2"/>
-      <c r="E15" s="2"/>
+      <c r="C2" s="11" t="s">
+        <v>15</v>
+      </c>
+      <c r="D2" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="F2" s="2"/>
+      <c r="G2" s="2"/>
+      <c r="H2" s="6"/>
+    </row>
+    <row r="3" spans="1:8" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A3" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="C3" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="D3" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="F3" s="2"/>
+      <c r="G3" s="2"/>
+      <c r="H3" s="6"/>
+    </row>
+    <row r="4" spans="1:8" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A4" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="C4" s="11" t="s">
+        <v>18</v>
+      </c>
+      <c r="D4" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="F4" s="2"/>
+      <c r="G4" s="2"/>
+      <c r="H4" s="6"/>
+    </row>
+    <row r="5" spans="1:8" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A5" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="C5" s="11" t="s">
+        <v>15</v>
+      </c>
+      <c r="D5" s="10" t="s">
+        <v>19</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="F5" s="2"/>
+      <c r="G5" s="2"/>
+      <c r="H5" s="2"/>
+    </row>
+    <row r="6" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="C6" s="10"/>
+      <c r="D6" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="F6" s="2"/>
+      <c r="G6" s="2"/>
+      <c r="H6" s="2"/>
+    </row>
+    <row r="7" spans="1:8" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A7" s="8" t="s">
+        <v>25</v>
+      </c>
+      <c r="B7" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="C7" s="11" t="s">
+        <v>15</v>
+      </c>
+      <c r="D7" s="10"/>
+      <c r="E7" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="F7" s="2"/>
+      <c r="G7" s="2"/>
+      <c r="H7" s="2"/>
+    </row>
+    <row r="8" spans="1:8" ht="43.8" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="C8" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="D8" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="F8" s="2"/>
+      <c r="G8" s="2"/>
+      <c r="H8" s="2"/>
+    </row>
+    <row r="9" spans="1:8" ht="42" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="B9" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="C9" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="D9" s="10" t="s">
+        <v>33</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="F9" s="2"/>
+      <c r="G9" s="2"/>
+      <c r="H9" s="2"/>
+    </row>
+    <row r="10" spans="1:8" ht="28.2" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="B10" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="C10" s="9"/>
+      <c r="D10" s="10"/>
+      <c r="E10" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="F10" s="2"/>
+      <c r="G10" s="2"/>
+      <c r="H10" s="2"/>
+    </row>
+    <row r="11" spans="1:8" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A11" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="B11" s="13" t="s">
+        <v>36</v>
+      </c>
+      <c r="C11" s="14" t="s">
+        <v>37</v>
+      </c>
+      <c r="D11" s="15" t="s">
+        <v>12</v>
+      </c>
+      <c r="E11" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="F11" s="2"/>
+      <c r="G11" s="2"/>
+      <c r="H11" s="2"/>
+    </row>
+    <row r="12" spans="1:8" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A12" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="C12" s="11" t="s">
+        <v>15</v>
+      </c>
+      <c r="D12" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="F12" s="2"/>
+      <c r="G12" s="2"/>
+      <c r="H12" s="2"/>
+    </row>
+    <row r="13" spans="1:8" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A13" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="B13" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="C13" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="D13" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="E13" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="F13" s="2"/>
+      <c r="G13" s="2"/>
+      <c r="H13" s="2"/>
+    </row>
+    <row r="14" spans="1:8" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A14" s="8" t="s">
+        <v>40</v>
+      </c>
+      <c r="B14" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="C14" s="11" t="s">
+        <v>18</v>
+      </c>
+      <c r="D14" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="E14" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="F14" s="2"/>
+      <c r="G14" s="2"/>
+      <c r="H14" s="2"/>
+    </row>
+    <row r="15" spans="1:8" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A15" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="B15" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="C15" s="11" t="s">
+        <v>15</v>
+      </c>
+      <c r="D15" s="10" t="s">
+        <v>19</v>
+      </c>
+      <c r="E15" s="2" t="s">
+        <v>34</v>
+      </c>
       <c r="F15" s="2"/>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A16" s="2"/>
-      <c r="B16" s="2"/>
-      <c r="C16" s="2"/>
-      <c r="D16" s="2"/>
-      <c r="E16" s="2"/>
+      <c r="G15" s="2"/>
+      <c r="H15" s="2"/>
+    </row>
+    <row r="16" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="8" t="s">
+        <v>42</v>
+      </c>
+      <c r="B16" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="C16" s="10"/>
+      <c r="D16" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="E16" s="2" t="s">
+        <v>34</v>
+      </c>
       <c r="F16" s="2"/>
+      <c r="G16" s="2"/>
+      <c r="H16" s="2"/>
+    </row>
+    <row r="17" spans="1:8" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A17" s="8" t="s">
+        <v>43</v>
+      </c>
+      <c r="B17" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="C17" s="11" t="s">
+        <v>15</v>
+      </c>
+      <c r="D17" s="10"/>
+      <c r="E17" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="F17" s="2"/>
+      <c r="G17" s="2"/>
+      <c r="H17" s="2"/>
+    </row>
+    <row r="18" spans="1:8" ht="43.8" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="8" t="s">
+        <v>44</v>
+      </c>
+      <c r="B18" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="C18" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="D18" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="E18" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="F18" s="2"/>
+      <c r="G18" s="2"/>
+      <c r="H18" s="2"/>
+    </row>
+    <row r="19" spans="1:8" ht="42" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A19" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="B19" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="C19" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="D19" s="10" t="s">
+        <v>33</v>
+      </c>
+      <c r="E19" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="F19" s="2"/>
+      <c r="G19" s="2"/>
+      <c r="H19" s="2"/>
+    </row>
+    <row r="20" spans="1:8" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A20" s="8" t="s">
+        <v>46</v>
+      </c>
+      <c r="B20" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="C20" s="9"/>
+      <c r="D20" s="2"/>
+      <c r="E20" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="F20" s="2"/>
+      <c r="G20" s="2"/>
+      <c r="H20" s="2"/>
     </row>
   </sheetData>
+  <phoneticPr fontId="5" type="noConversion"/>
+  <hyperlinks>
+    <hyperlink ref="C2" r:id="rId1" xr:uid="{E82F255B-1660-4B9C-82D0-B191BA758285}"/>
+    <hyperlink ref="C3" r:id="rId2" xr:uid="{3A826DDE-60C7-4AF9-959A-635B5EB020BE}"/>
+    <hyperlink ref="C4" r:id="rId3" xr:uid="{CCE2EA27-DBAE-4584-946A-D5C1994C6936}"/>
+    <hyperlink ref="C5" r:id="rId4" xr:uid="{ECFCD4C9-FB87-401F-9C22-F0882AF0FE45}"/>
+    <hyperlink ref="C7" r:id="rId5" xr:uid="{C3A083D9-B22F-446E-A2F1-7A525C5F7724}"/>
+    <hyperlink ref="C8" r:id="rId6" xr:uid="{9F6A08AE-9FD7-4FD7-813C-FED3A8184BF4}"/>
+    <hyperlink ref="C9" r:id="rId7" xr:uid="{FCBADB3D-A359-43CB-96B8-FF5BEBC27D2F}"/>
+    <hyperlink ref="C12" r:id="rId8" xr:uid="{6202DCD7-0689-4C9B-A379-0E93B9037508}"/>
+    <hyperlink ref="C13" r:id="rId9" xr:uid="{CBF8E205-3FC5-4C6D-8D88-984C8782F71C}"/>
+    <hyperlink ref="C14" r:id="rId10" xr:uid="{5C692B60-6AB1-44E2-B091-9578AA47FB33}"/>
+    <hyperlink ref="C15" r:id="rId11" xr:uid="{02DE5336-CF06-4656-BB23-609039868458}"/>
+    <hyperlink ref="C17" r:id="rId12" xr:uid="{4E246B45-84E3-4350-BF34-FE04D281D0E4}"/>
+    <hyperlink ref="C18" r:id="rId13" xr:uid="{5A69D364-3A2F-44E5-B2B8-074A69081BAF}"/>
+    <hyperlink ref="C19" r:id="rId14" xr:uid="{4BE6AA11-F89D-4F5C-BE0A-D662242A7640}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId1"/>
+  <pageSetup orientation="portrait" r:id="rId15"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: test script app
</commit_message>
<xml_diff>
--- a/data/data_test.xlsx
+++ b/data/data_test.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="25601"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24026"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Test\script-test\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3D37CC93-7C75-42D6-AB59-45EA633E4A4A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6ED913A8-96F6-45A2-9466-1E84CCD669A6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{8FAFAB84-7321-4A60-AD43-F6BDBFF31D96}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20640" windowHeight="11160" xr2:uid="{8FAFAB84-7321-4A60-AD43-F6BDBFF31D96}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="95" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="95" uniqueCount="49">
   <si>
     <t>Test Case ID</t>
   </si>
@@ -175,6 +175,12 @@
   </si>
   <si>
     <t>[Login-30]</t>
+  </si>
+  <si>
+    <t>tranguyenvannhut@gmail.com</t>
+  </si>
+  <si>
+    <t>8di0ha66</t>
   </si>
 </sst>
 </file>
@@ -694,18 +700,18 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A869C040-2518-4127-9479-80AA9CA67B0C}">
   <dimension ref="A1:H20"/>
-  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="11.5546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="28.88671875" style="1" customWidth="1"/>
-    <col min="3" max="3" width="35.5546875" style="1" customWidth="1"/>
-    <col min="4" max="4" width="25.6640625" style="1" customWidth="1"/>
-    <col min="5" max="5" width="23.88671875" style="1" customWidth="1"/>
-    <col min="6" max="6" width="18.33203125" style="1" customWidth="1"/>
-    <col min="7" max="16384" width="9.109375" style="1"/>
+    <col min="1" max="1" width="11.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="28.85546875" style="1" customWidth="1"/>
+    <col min="3" max="3" width="35.5703125" style="1" customWidth="1"/>
+    <col min="4" max="4" width="25.7109375" style="1" customWidth="1"/>
+    <col min="5" max="5" width="23.85546875" style="1" customWidth="1"/>
+    <col min="6" max="6" width="18.28515625" style="1" customWidth="1"/>
+    <col min="7" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:8" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -731,7 +737,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:8" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="7" t="s">
         <v>20</v>
       </c>
@@ -739,10 +745,10 @@
         <v>5</v>
       </c>
       <c r="C2" s="11" t="s">
-        <v>15</v>
+        <v>47</v>
       </c>
       <c r="D2" s="10" t="s">
-        <v>16</v>
+        <v>48</v>
       </c>
       <c r="E2" s="2" t="s">
         <v>14</v>
@@ -751,7 +757,7 @@
       <c r="G2" s="2"/>
       <c r="H2" s="6"/>
     </row>
-    <row r="3" spans="1:8" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:8" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="8" t="s">
         <v>21</v>
       </c>
@@ -771,7 +777,7 @@
       <c r="G3" s="2"/>
       <c r="H3" s="6"/>
     </row>
-    <row r="4" spans="1:8" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:8" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="8" t="s">
         <v>22</v>
       </c>
@@ -791,7 +797,7 @@
       <c r="G4" s="2"/>
       <c r="H4" s="6"/>
     </row>
-    <row r="5" spans="1:8" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:8" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="8" t="s">
         <v>23</v>
       </c>
@@ -811,7 +817,7 @@
       <c r="G5" s="2"/>
       <c r="H5" s="2"/>
     </row>
-    <row r="6" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:8" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="8" t="s">
         <v>24</v>
       </c>
@@ -829,7 +835,7 @@
       <c r="G6" s="2"/>
       <c r="H6" s="2"/>
     </row>
-    <row r="7" spans="1:8" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:8" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" s="8" t="s">
         <v>25</v>
       </c>
@@ -847,7 +853,7 @@
       <c r="G7" s="2"/>
       <c r="H7" s="2"/>
     </row>
-    <row r="8" spans="1:8" ht="43.8" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:8" ht="45.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="8" t="s">
         <v>26</v>
       </c>
@@ -867,7 +873,7 @@
       <c r="G8" s="2"/>
       <c r="H8" s="2"/>
     </row>
-    <row r="9" spans="1:8" ht="42" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:8" ht="45.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="8" t="s">
         <v>27</v>
       </c>
@@ -887,7 +893,7 @@
       <c r="G9" s="2"/>
       <c r="H9" s="2"/>
     </row>
-    <row r="10" spans="1:8" ht="28.2" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:8" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="8" t="s">
         <v>28</v>
       </c>
@@ -903,7 +909,7 @@
       <c r="G10" s="2"/>
       <c r="H10" s="2"/>
     </row>
-    <row r="11" spans="1:8" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:8" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="7" t="s">
         <v>35</v>
       </c>
@@ -923,7 +929,7 @@
       <c r="G11" s="2"/>
       <c r="H11" s="2"/>
     </row>
-    <row r="12" spans="1:8" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:8" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="7" t="s">
         <v>38</v>
       </c>
@@ -943,7 +949,7 @@
       <c r="G12" s="2"/>
       <c r="H12" s="2"/>
     </row>
-    <row r="13" spans="1:8" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:8" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A13" s="8" t="s">
         <v>39</v>
       </c>
@@ -963,7 +969,7 @@
       <c r="G13" s="2"/>
       <c r="H13" s="2"/>
     </row>
-    <row r="14" spans="1:8" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:8" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A14" s="8" t="s">
         <v>40</v>
       </c>
@@ -983,7 +989,7 @@
       <c r="G14" s="2"/>
       <c r="H14" s="2"/>
     </row>
-    <row r="15" spans="1:8" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:8" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A15" s="8" t="s">
         <v>41</v>
       </c>
@@ -1003,7 +1009,7 @@
       <c r="G15" s="2"/>
       <c r="H15" s="2"/>
     </row>
-    <row r="16" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:8" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="8" t="s">
         <v>42</v>
       </c>
@@ -1021,7 +1027,7 @@
       <c r="G16" s="2"/>
       <c r="H16" s="2"/>
     </row>
-    <row r="17" spans="1:8" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:8" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="8" t="s">
         <v>43</v>
       </c>
@@ -1039,7 +1045,7 @@
       <c r="G17" s="2"/>
       <c r="H17" s="2"/>
     </row>
-    <row r="18" spans="1:8" ht="43.8" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:8" ht="45.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A18" s="8" t="s">
         <v>44</v>
       </c>
@@ -1059,7 +1065,7 @@
       <c r="G18" s="2"/>
       <c r="H18" s="2"/>
     </row>
-    <row r="19" spans="1:8" ht="42" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:8" ht="45.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A19" s="8" t="s">
         <v>45</v>
       </c>
@@ -1079,7 +1085,7 @@
       <c r="G19" s="2"/>
       <c r="H19" s="2"/>
     </row>
-    <row r="20" spans="1:8" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:8" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A20" s="8" t="s">
         <v>46</v>
       </c>

</xml_diff>

<commit_message>
Fix: test-login, Feat: test-register
</commit_message>
<xml_diff>
--- a/data/data_test.xlsx
+++ b/data/data_test.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="25601"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Test\script-test\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\nam3\KTPM2\Script-test-ecommerece\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6ED913A8-96F6-45A2-9466-1E84CCD669A6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{02972552-08FD-4AB1-A83B-5F5F3A836970}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20640" windowHeight="11160" xr2:uid="{8FAFAB84-7321-4A60-AD43-F6BDBFF31D96}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{8FAFAB84-7321-4A60-AD43-F6BDBFF31D96}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="95" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="62">
   <si>
     <t>Test Case ID</t>
   </si>
@@ -144,9 +144,6 @@
     <t>[Login-21]</t>
   </si>
   <si>
-    <t>Test login with an incorrectly formatted email</t>
-  </si>
-  <si>
     <t>testuserexample.com</t>
   </si>
   <si>
@@ -177,10 +174,56 @@
     <t>[Login-30]</t>
   </si>
   <si>
-    <t>tranguyenvannhut@gmail.com</t>
-  </si>
-  <si>
-    <t>8di0ha66</t>
+    <t xml:space="preserve">	testuser@example.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">	Password123</t>
+  </si>
+  <si>
+    <t>wrongemail@example.com</t>
+  </si>
+  <si>
+    <t>Navigate to home screen</t>
+  </si>
+  <si>
+    <t>Alert: "Invalid email or password!"
+Stay on login</t>
+  </si>
+  <si>
+    <t>Pass</t>
+  </si>
+  <si>
+    <t xml:space="preserve">	Password less than 6 characters</t>
+  </si>
+  <si>
+    <t>Test login with missing email</t>
+  </si>
+  <si>
+    <t>Test login with missing password</t>
+  </si>
+  <si>
+    <t>Invalid email format</t>
+  </si>
+  <si>
+    <t>invalidemail</t>
+  </si>
+  <si>
+    <t>Test login with invalid email</t>
+  </si>
+  <si>
+    <t xml:space="preserve">	Test login with valid credentials</t>
+  </si>
+  <si>
+    <t>Alert: "Password must be at least 6 characters long!"
+Stay on login</t>
+  </si>
+  <si>
+    <t xml:space="preserve">	Alert: "Please enter both email and password!"
+Stay on login</t>
+  </si>
+  <si>
+    <t xml:space="preserve">	Alert: "Invalid email format"
+Stay on login</t>
   </si>
 </sst>
 </file>
@@ -699,19 +742,19 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A869C040-2518-4127-9479-80AA9CA67B0C}">
-  <dimension ref="A1:H20"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:H36"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="11.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="28.85546875" style="1" customWidth="1"/>
-    <col min="3" max="3" width="35.5703125" style="1" customWidth="1"/>
-    <col min="4" max="4" width="25.7109375" style="1" customWidth="1"/>
-    <col min="5" max="5" width="23.85546875" style="1" customWidth="1"/>
-    <col min="6" max="6" width="18.28515625" style="1" customWidth="1"/>
-    <col min="7" max="16384" width="9.140625" style="1"/>
+    <col min="1" max="1" width="11.5546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="28.88671875" style="1" customWidth="1"/>
+    <col min="3" max="3" width="35.5546875" style="1" customWidth="1"/>
+    <col min="4" max="4" width="25.6640625" style="1" customWidth="1"/>
+    <col min="5" max="5" width="23.88671875" style="1" customWidth="1"/>
+    <col min="6" max="6" width="20.88671875" style="1" customWidth="1"/>
+    <col min="7" max="16384" width="9.109375" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -737,35 +780,37 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" s="7" t="s">
         <v>20</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>5</v>
+        <v>58</v>
       </c>
       <c r="C2" s="11" t="s">
+        <v>46</v>
+      </c>
+      <c r="D2" s="10" t="s">
         <v>47</v>
-      </c>
-      <c r="D2" s="10" t="s">
-        <v>48</v>
       </c>
       <c r="E2" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="F2" s="2"/>
+      <c r="F2" t="s">
+        <v>49</v>
+      </c>
       <c r="G2" s="2"/>
       <c r="H2" s="6"/>
     </row>
-    <row r="3" spans="1:8" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8" ht="42" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A3" s="8" t="s">
         <v>21</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>6</v>
+        <v>57</v>
       </c>
       <c r="C3" s="11" t="s">
-        <v>17</v>
+        <v>48</v>
       </c>
       <c r="D3" s="10" t="s">
         <v>16</v>
@@ -773,165 +818,156 @@
       <c r="E3" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="F3" s="2"/>
+      <c r="F3" s="2" t="s">
+        <v>50</v>
+      </c>
       <c r="G3" s="2"/>
       <c r="H3" s="6"/>
     </row>
-    <row r="4" spans="1:8" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:8" ht="42" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A4" s="8" t="s">
         <v>22</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C4" s="11" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="D4" s="10" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="E4" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="F4" s="2"/>
+      <c r="F4" s="2" t="s">
+        <v>50</v>
+      </c>
       <c r="G4" s="2"/>
       <c r="H4" s="6"/>
     </row>
-    <row r="5" spans="1:8" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:8" ht="55.8" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A5" s="8" t="s">
         <v>23</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>8</v>
+        <v>52</v>
       </c>
       <c r="C5" s="11" t="s">
         <v>15</v>
       </c>
       <c r="D5" s="10" t="s">
-        <v>19</v>
+        <v>51</v>
       </c>
       <c r="E5" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="F5" s="2"/>
+      <c r="F5" s="2" t="s">
+        <v>59</v>
+      </c>
       <c r="G5" s="2"/>
       <c r="H5" s="2"/>
     </row>
-    <row r="6" spans="1:8" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:8" ht="55.8" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A6" s="8" t="s">
         <v>24</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="C6" s="10"/>
-      <c r="D6" s="10" t="s">
-        <v>16</v>
-      </c>
+        <v>10</v>
+      </c>
+      <c r="C6" s="11" t="s">
+        <v>15</v>
+      </c>
+      <c r="D6" s="10"/>
       <c r="E6" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="F6" s="2"/>
+      <c r="F6" s="2" t="s">
+        <v>60</v>
+      </c>
       <c r="G6" s="2"/>
       <c r="H6" s="2"/>
     </row>
-    <row r="7" spans="1:8" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:8" ht="42" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" s="8" t="s">
         <v>25</v>
       </c>
-      <c r="B7" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="C7" s="11" t="s">
-        <v>15</v>
-      </c>
-      <c r="D7" s="10"/>
+      <c r="B7" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="C7" s="12"/>
+      <c r="D7" s="10" t="s">
+        <v>16</v>
+      </c>
       <c r="E7" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="F7" s="2"/>
+      <c r="F7" s="2" t="s">
+        <v>61</v>
+      </c>
       <c r="G7" s="2"/>
       <c r="H7" s="2"/>
     </row>
-    <row r="8" spans="1:8" ht="45.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:8" ht="28.2" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="8" t="s">
         <v>26</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>29</v>
+        <v>54</v>
       </c>
       <c r="C8" s="12" t="s">
-        <v>32</v>
-      </c>
-      <c r="D8" s="10" t="s">
-        <v>16</v>
-      </c>
-      <c r="E8" s="2" t="s">
-        <v>14</v>
-      </c>
+        <v>15</v>
+      </c>
+      <c r="D8" s="10"/>
+      <c r="E8" s="2"/>
       <c r="F8" s="2"/>
       <c r="G8" s="2"/>
       <c r="H8" s="2"/>
     </row>
-    <row r="9" spans="1:8" ht="45.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="B9" s="5" t="s">
-        <v>30</v>
-      </c>
-      <c r="C9" s="12" t="s">
-        <v>15</v>
-      </c>
-      <c r="D9" s="10" t="s">
-        <v>33</v>
-      </c>
-      <c r="E9" s="2" t="s">
-        <v>14</v>
-      </c>
+      <c r="B9" s="13" t="s">
+        <v>55</v>
+      </c>
+      <c r="C9" s="9" t="s">
+        <v>56</v>
+      </c>
+      <c r="D9" s="10"/>
+      <c r="E9" s="2"/>
       <c r="F9" s="2"/>
       <c r="G9" s="2"/>
       <c r="H9" s="2"/>
     </row>
-    <row r="10" spans="1:8" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A10" s="8" t="s">
         <v>28</v>
       </c>
-      <c r="B10" s="5" t="s">
-        <v>31</v>
-      </c>
-      <c r="C10" s="9"/>
-      <c r="D10" s="10"/>
-      <c r="E10" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="F10" s="2"/>
       <c r="G10" s="2"/>
       <c r="H10" s="2"/>
     </row>
-    <row r="11" spans="1:8" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A11" s="7" t="s">
         <v>35</v>
       </c>
       <c r="B11" s="13" t="s">
+        <v>55</v>
+      </c>
+      <c r="C11" s="14" t="s">
         <v>36</v>
-      </c>
-      <c r="C11" s="14" t="s">
-        <v>37</v>
       </c>
       <c r="D11" s="15" t="s">
         <v>12</v>
       </c>
-      <c r="E11" s="2" t="s">
-        <v>14</v>
-      </c>
+      <c r="E11" s="2"/>
       <c r="F11" s="2"/>
       <c r="G11" s="2"/>
       <c r="H11" s="2"/>
     </row>
-    <row r="12" spans="1:8" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:8" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A12" s="7" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B12" s="4" t="s">
         <v>5</v>
@@ -949,9 +985,9 @@
       <c r="G12" s="2"/>
       <c r="H12" s="2"/>
     </row>
-    <row r="13" spans="1:8" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:8" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A13" s="8" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B13" s="5" t="s">
         <v>6</v>
@@ -969,9 +1005,9 @@
       <c r="G13" s="2"/>
       <c r="H13" s="2"/>
     </row>
-    <row r="14" spans="1:8" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:8" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A14" s="8" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B14" s="5" t="s">
         <v>7</v>
@@ -989,9 +1025,9 @@
       <c r="G14" s="2"/>
       <c r="H14" s="2"/>
     </row>
-    <row r="15" spans="1:8" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:8" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A15" s="8" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B15" s="5" t="s">
         <v>8</v>
@@ -1009,9 +1045,9 @@
       <c r="G15" s="2"/>
       <c r="H15" s="2"/>
     </row>
-    <row r="16" spans="1:8" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="8" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B16" s="5" t="s">
         <v>9</v>
@@ -1027,9 +1063,9 @@
       <c r="G16" s="2"/>
       <c r="H16" s="2"/>
     </row>
-    <row r="17" spans="1:8" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:8" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A17" s="8" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B17" s="5" t="s">
         <v>10</v>
@@ -1045,9 +1081,9 @@
       <c r="G17" s="2"/>
       <c r="H17" s="2"/>
     </row>
-    <row r="18" spans="1:8" ht="45.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:8" ht="43.8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A18" s="8" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B18" s="4" t="s">
         <v>29</v>
@@ -1065,9 +1101,9 @@
       <c r="G18" s="2"/>
       <c r="H18" s="2"/>
     </row>
-    <row r="19" spans="1:8" ht="45.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:8" ht="42" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A19" s="8" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B19" s="5" t="s">
         <v>30</v>
@@ -1085,9 +1121,9 @@
       <c r="G19" s="2"/>
       <c r="H19" s="2"/>
     </row>
-    <row r="20" spans="1:8" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:8" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A20" s="8" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B20" s="5" t="s">
         <v>31</v>
@@ -1101,25 +1137,42 @@
       <c r="G20" s="2"/>
       <c r="H20" s="2"/>
     </row>
+    <row r="35" spans="3:4" ht="43.2" x14ac:dyDescent="0.25">
+      <c r="C35" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="D35" s="10" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="36" spans="3:4" ht="41.4" x14ac:dyDescent="0.25">
+      <c r="C36" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="D36" s="10" t="s">
+        <v>33</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="5" type="noConversion"/>
   <hyperlinks>
-    <hyperlink ref="C2" r:id="rId1" xr:uid="{E82F255B-1660-4B9C-82D0-B191BA758285}"/>
+    <hyperlink ref="C2" r:id="rId1" display="tranguyenvannhut@gmail.com" xr:uid="{E82F255B-1660-4B9C-82D0-B191BA758285}"/>
     <hyperlink ref="C3" r:id="rId2" xr:uid="{3A826DDE-60C7-4AF9-959A-635B5EB020BE}"/>
-    <hyperlink ref="C4" r:id="rId3" xr:uid="{CCE2EA27-DBAE-4584-946A-D5C1994C6936}"/>
-    <hyperlink ref="C5" r:id="rId4" xr:uid="{ECFCD4C9-FB87-401F-9C22-F0882AF0FE45}"/>
-    <hyperlink ref="C7" r:id="rId5" xr:uid="{C3A083D9-B22F-446E-A2F1-7A525C5F7724}"/>
-    <hyperlink ref="C8" r:id="rId6" xr:uid="{9F6A08AE-9FD7-4FD7-813C-FED3A8184BF4}"/>
-    <hyperlink ref="C9" r:id="rId7" xr:uid="{FCBADB3D-A359-43CB-96B8-FF5BEBC27D2F}"/>
-    <hyperlink ref="C12" r:id="rId8" xr:uid="{6202DCD7-0689-4C9B-A379-0E93B9037508}"/>
-    <hyperlink ref="C13" r:id="rId9" xr:uid="{CBF8E205-3FC5-4C6D-8D88-984C8782F71C}"/>
-    <hyperlink ref="C14" r:id="rId10" xr:uid="{5C692B60-6AB1-44E2-B091-9578AA47FB33}"/>
-    <hyperlink ref="C15" r:id="rId11" xr:uid="{02DE5336-CF06-4656-BB23-609039868458}"/>
-    <hyperlink ref="C17" r:id="rId12" xr:uid="{4E246B45-84E3-4350-BF34-FE04D281D0E4}"/>
-    <hyperlink ref="C18" r:id="rId13" xr:uid="{5A69D364-3A2F-44E5-B2B8-074A69081BAF}"/>
-    <hyperlink ref="C19" r:id="rId14" xr:uid="{4BE6AA11-F89D-4F5C-BE0A-D662242A7640}"/>
+    <hyperlink ref="C6" r:id="rId3" xr:uid="{C3A083D9-B22F-446E-A2F1-7A525C5F7724}"/>
+    <hyperlink ref="C8" r:id="rId4" xr:uid="{FCBADB3D-A359-43CB-96B8-FF5BEBC27D2F}"/>
+    <hyperlink ref="C12" r:id="rId5" xr:uid="{6202DCD7-0689-4C9B-A379-0E93B9037508}"/>
+    <hyperlink ref="C13" r:id="rId6" xr:uid="{CBF8E205-3FC5-4C6D-8D88-984C8782F71C}"/>
+    <hyperlink ref="C14" r:id="rId7" xr:uid="{5C692B60-6AB1-44E2-B091-9578AA47FB33}"/>
+    <hyperlink ref="C15" r:id="rId8" xr:uid="{02DE5336-CF06-4656-BB23-609039868458}"/>
+    <hyperlink ref="C17" r:id="rId9" xr:uid="{4E246B45-84E3-4350-BF34-FE04D281D0E4}"/>
+    <hyperlink ref="C18" r:id="rId10" xr:uid="{5A69D364-3A2F-44E5-B2B8-074A69081BAF}"/>
+    <hyperlink ref="C19" r:id="rId11" xr:uid="{4BE6AA11-F89D-4F5C-BE0A-D662242A7640}"/>
+    <hyperlink ref="C5" r:id="rId12" xr:uid="{EF50CC98-4457-4FA1-A90F-3B28D629760D}"/>
+    <hyperlink ref="C4" r:id="rId13" xr:uid="{ECFCD4C9-FB87-401F-9C22-F0882AF0FE45}"/>
+    <hyperlink ref="C35" r:id="rId14" xr:uid="{56EEC0AA-9457-4E85-BB45-F1F2DCE48E8B}"/>
+    <hyperlink ref="C36" r:id="rId15" xr:uid="{5D067DBD-F10F-4CD8-8BC6-05978E8A5545}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId15"/>
+  <pageSetup orientation="portrait" r:id="rId16"/>
 </worksheet>
 </file>
</xml_diff>